<commit_message>
Record first 8 many-analyst studies with organizer contacts
Adds Huntington-Klein 2021, HK&Portner 2026, Silberzahn 2018, Schweinsberg
2021, Breznau 2022, Landy 2020, Botvinik-Nezer/NARPS 2020, and Menkveld
Nonstandard Errors 2024 (with organizing committee) to Contact Info.xlsx.
Updates queue and progress log.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +453,758 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Huntington-Klein et al. (2021) - The Influence of Hidden Researcher Decisions in Applied Microeconomics</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/ecin.12992</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nick Huntington-Klein</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nhuntington-klein@seattleu.edu</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+1 (206) 296-5815</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Department of Economics, Seattle University, Seattle, WA, USA</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Lead/corresponding author &amp; project organizer. Economic Inquiry 59(3):944-960. Seven replicators x two econ studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Huntington-Klein &amp; Portner (2026) - The Sources of Researcher Variation in Economics (Many-Economists)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17605/OSF.IO/CJ9YX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nick Huntington-Klein</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nhuntington-klein@seattleu.edu</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+1 (206) 296-5815</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Department of Economics, Seattle University, Seattle, WA, USA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Co-organizer (corresponding author). Forthcoming JEL. 146 research teams. Project: Many Economists Collaborative on Researcher Variation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Huntington-Klein &amp; Portner (2026) - The Sources of Researcher Variation in Economics (Many-Economists)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17605/OSF.IO/CJ9YX</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Claus C. Portner</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>cportner@seattleu.edu</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Department of Economics, Albers School of Business and Economics, Seattle University, Seattle, WA, USA</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Co-organizer. Also affiliated with Center for Studies in Demography and Ecology, Univ. of Washington. Personal site clausportner.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Silberzahn et al. (2018) - Many Analysts, One Data Set</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/2515245917747646</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Raphael Silberzahn</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>r.silberzahn@gmail.com</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>University of Sussex Business School, Brighton, UK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Co-lead organizer. Adv Methods Practices Psych Sci 1(3):337-356. 29 teams analyzed soccer referee skin-tone/red-card data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Silberzahn et al. (2018) - Many Analysts, One Data Set</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/2515245917747646</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Eric Luis Uhlmann</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>eric.luis.uhlmann@gmail.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>INSEAD, Singapore</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Co-lead/senior organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Schweinsberg et al. (2021) - Same Data, Different Conclusions</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.obhdp.2021.02.003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Martin Schweinsberg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>martin.schweinsberg@esmt.org</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ESMT Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Lead organizer. OBHDP 165:228-249. Crowdsourcing data analysis project (DataExplained).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Schweinsberg et al. (2021) - Same Data, Different Conclusions</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.obhdp.2021.02.003</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Eric Luis Uhlmann</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>eric.luis.uhlmann@gmail.com</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>INSEAD, Singapore</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Senior/co-organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Breznau et al. (2022) - Observing Many Researchers Using the Same Data and Hypothesis Reveals a Hidden Universe of Uncertainty</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2203150119</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nate Breznau</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>breznau.nate@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+49 421-218-58644</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SOCIUM Research Center on Inequality and Social Policy, University of Bremen, Germany</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Lead organizer (CRI / Crowdsourced Replication Initiative). PNAS 119(44). 73 teams, immigration &amp; social policy support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Breznau et al. (2022) - Observing Many Researchers Using the Same Data and Hypothesis Reveals a Hidden Universe of Uncertainty</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2203150119</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Eike Mark Rinke</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>University of Leeds, UK (School of Politics and International Studies)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Co-organizer. Email to be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Breznau et al. (2022) - Observing Many Researchers Using the Same Data and Hypothesis Reveals a Hidden Universe of Uncertainty</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2203150119</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Alexander Wuttke</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LMU Munich, Germany (Political Science)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Co-organizer. Email to be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Landy et al. (2020) - Crowdsourcing Hypothesis Tests</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/bul0000220</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Justin F. Landy</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Nova Southeastern University, FL, USA (Dept. of Psychology)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Lead author. Psychological Bulletin 146(5):451-479. 15 teams designed studies for 5 hypotheses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Landy et al. (2020) - Crowdsourcing Hypothesis Tests</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/bul0000220</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Eric Luis Uhlmann</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>eric.luis.uhlmann@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>INSEAD, Singapore</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Senior organizer (corresponding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Botvinik-Nezer et al. (2020) - Variability in the Analysis of a Single Neuroimaging Dataset by Many Teams (NARPS)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-020-2314-9</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rotem Botvinik-Nezer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Sagol School of Neuroscience, Tel Aviv University (at time of study); later Dartmouth College / Technion</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Lead organizer of NARPS. Nature 582:84-88. 70 teams analyzed fMRI mixed-gamble data, 9 hypotheses. Email to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Botvinik-Nezer et al. (2020) - Variability in the Analysis of a Single Neuroimaging Dataset by Many Teams (NARPS)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-020-2314-9</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tom Schonberg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>schonberg@tauex.tau.ac.il</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sagol School of Neuroscience &amp; School of Neurobiology, Tel Aviv University, Israel</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Corresponding author / senior organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Botvinik-Nezer et al. (2020) - Variability in the Analysis of a Single Neuroimaging Dataset by Many Teams (NARPS)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-020-2314-9</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Russell A. Poldrack</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>russpold@stanford.edu</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Department of Psychology, Stanford University, CA, USA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Corresponding author / senior organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Albert J. Menkveld</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>a.j.menkveld@vu.nl</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>School of Business and Economics, Vrije Universiteit Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Lead organizer. Journal of Finance 79(3):2339-2390. 164 teams test 6 finance hypotheses on same data. Organizing committee = first 8 authors (Menkveld, Dreber, Holzmeister, Huber, Johannesson, Kirchler, Razen, Weitzel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Anna Dreber</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>anna.dreber@hhs.se</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Department of Economics, Stockholm School of Economics, Sweden</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Felix Holzmeister</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>felix.holzmeister@uibk.ac.at</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Department of Economics, University of Innsbruck, Austria</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Juergen Huber</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>juergen.huber@uibk.ac.at</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Department of Banking and Finance, University of Innsbruck, Austria</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Magnus Johannesson</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>magnus.johannesson@hhs.se</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Department of Economics, Stockholm School of Economics, Sweden</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Michael Kirchler</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>michael.kirchler@uibk.ac.at</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Department of Banking and Finance, University of Innsbruck, Austria</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Michael Razen</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>University of Innsbruck, Austria (at time of study)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator. Email to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Menkveld et al. (2024) - Nonstandard Errors</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jofi.13337</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Utz Weitzel</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>u.weitzel@vu.nl</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>School of Business and Economics, Vrije Universiteit Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record Hoogeveen/MARP, Gould, Ostropolets, Bastiaansen; file Holzmeister 2024 as inappropriate
Adds religiosity-wellbeing MARP, ecology same-data, OHDSI reproducibility,
and ESM treatment-target many-analyst studies. Files Holzmeister 2024 as a
synthesis paper. Enqueues the 45-team Competition and Moral Behavior study.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1193,7 +1193,6 @@
           <t>u.weitzel@vu.nl</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>School of Business and Economics, Vrije Universiteit Amsterdam, Netherlands</t>
@@ -1202,6 +1201,327 @@
       <c r="G24" t="inlineStr">
         <is>
           <t>Organizing committee / research coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hoogeveen et al. (2023) - A Many-Analysts Approach to the Relation between Religiosity and Well-being (MARP)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/2153599X.2022.2070255</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Suzanne Hoogeveen</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>suzanne.j.hoogeveen@gmail.com</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Department of Psychology, University of Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Lead organizer, Many-Analysts Religion Project (MARP). Religion Brain &amp; Behavior 13(3):237-283. 120+ analyst teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hoogeveen et al. (2023) - A Many-Analysts Approach to the Relation between Religiosity and Well-being (MARP)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/2153599X.2022.2070255</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Alexandra Sarafoglou</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>a.s.g.sarafoglou@uva.nl</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Department of Psychological Methods, University of Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Co-organizer, MARP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hoogeveen et al. (2023) - A Many-Analysts Approach to the Relation between Religiosity and Well-being (MARP)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/2153599X.2022.2070255</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Balazs Aczel</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>aczel.balazs@ppk.elte.hu</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Institute of Psychology, ELTE Eotvos Lorand University, Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Co-organizer / senior, MARP. Alt: balazs.aczel@gmail.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gould et al. (2025) - Same Data, Different Analysts: Variation in Effect Sizes (Ecology &amp; Evolutionary Biology)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12915-024-02101-x</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Elliot Gould</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>School of BioSciences, University of Melbourne, Australia</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Co-lead author/organizer (they/them). BMC Biology 23:35. 174 analysts/teams, 2 datasets. Email: unimelb.edu.au domain, exact unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Gould et al. (2025) - Same Data, Different Analysts: Variation in Effect Sizes (Ecology &amp; Evolutionary Biology)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12915-024-02101-x</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Hannah S. Fraser</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>School of BioSciences, University of Melbourne, Australia</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Co-lead author/organizer. Email unconfirmed (hannahsfraser@gmail.com likely).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Gould et al. (2025) - Same Data, Different Analysts: Variation in Effect Sizes (Ecology &amp; Evolutionary Biology)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12915-024-02101-x</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Timothy H. Parker</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>parkerth@whitman.edu</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Department of Biology, Whitman College, Walla Walla, WA, USA</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Corresponding/senior organizer (SORTEE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ostropolets et al. (2023) - Reproducible Variability: Investigator Discordance Across 9 Teams Reproducing the Same Observational Study</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/jamia/ocad009</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Anna Ostropolets</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Department of Biomedical Informatics, Columbia University Irving Medical Center, NY, USA (now Johnson &amp; Johnson)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Lead organizer (OHDSI). JAMIA 30(5):859-868. 9 teams reproduce same observational study. Email to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ostropolets et al. (2023) - Reproducible Variability: Investigator Discordance Across 9 Teams Reproducing the Same Observational Study</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/jamia/ocad009</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>George Hripcsak</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>hripcsak@columbia.edu</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Department of Biomedical Informatics, Columbia University, NY, USA</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Senior/corresponding organizer (OHDSI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bastiaansen et al. (2020) - Time to Get Personal? Impact of Researchers' Choices on Selection of Treatment Targets (ESM)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jpsychores.2020.110211</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Jojanneke A. Bastiaansen</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>j.a.bastiaansen@umcg.nl</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>University of Groningen, University Medical Center Groningen, Dept. of Psychiatry, Netherlands</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Lead organizer. J Psychosomatic Research 137:110211. 12 research labs analyzed one patient's ESM time-series. Email per UMCG pattern; verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Bastiaansen et al. (2020) - Time to Get Personal? Impact of Researchers' Choices on Selection of Treatment Targets (ESM)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jpsychores.2020.110211</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Laura F. Bringmann</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>l.f.bringmann@rug.nl</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Dept. of Psychometrics and Statistics, University of Groningen, Netherlands</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Senior/corresponding organizer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete seed-queue pass: 18 studies / 46 organizer rows
Records Dutilh 2019, Boehm 2018, Cohn 2016, Magnus & Morgan 1997, Ortloff
2023, and Huber 2023 (45 designs). Files Sulik 2023, Soebhag 2024, and
Sarafoglou 2024 as inappropriate. Queue emptied; PROGRESS updated to the
Google Scholar expansion pass with candidate leads.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1513,7 +1513,6 @@
           <t>l.f.bringmann@rug.nl</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Dept. of Psychometrics and Statistics, University of Groningen, Netherlands</t>
@@ -1522,6 +1521,423 @@
       <c r="G34" t="inlineStr">
         <is>
           <t>Senior/corresponding organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Dutilh et al. (2019) - The Quality of Response Time Data Inference: A Blinded, Collaborative Assessment of the Validity of Cognitive Models</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3758/s13423-017-1417-2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Gilles Dutilh</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Department of Psychology, University of Basel, Switzerland (now University Hospital Basel)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Lead organizer. Psychonomic Bulletin &amp; Review 26(4):1051-1069. 17 teams analyzed same 14 RT datasets, blinded. Email to verify (unibas.ch/usb.ch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Boehm et al. (2018) - Estimating Across-Trial Variability Parameters of the Diffusion Decision Model: Expert Advice and Recommendations</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmp.2018.09.004</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Udo Boehm</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Department of Psychology, University of Amsterdam / University of Groningen, Netherlands</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Lead organizer. J Mathematical Psychology 87:46-75. Multiple expert DDM teams each fit the same standardized data. Email to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Boehm et al. (2018) - Estimating Across-Trial Variability Parameters of the Diffusion Decision Model: Expert Advice and Recommendations</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmp.2018.09.004</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Eric-Jan Wagenmakers</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ej.wagenmakers@gmail.com</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Department of Psychological Methods, University of Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Senior organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cohn (2016) - We Gave Four Good Pollsters the Same Raw Data. They Had Four Different Results</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://www.nytimes.com/interactive/2016/09/20/upshot/the-error-the-polling-world-rarely-talks-about.html</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Nate Cohn</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>nate.cohn@nytimes.com</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>The New York Times (The Upshot), New York, NY, USA</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Journalistic many-analyst: 4 pollster teams analyzed the same 2016 Florida poll raw data. Organizer/author Nate Cohn. Email per NYT firstname.lastname@nytimes.com pattern; verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Magnus &amp; Morgan (1997) - The Experiment in Applied Econometrics (Tilburg Experiment: food demand / income elasticity)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/(SICI)1099-1255(199709/10)12:5&lt;459::AID-JAE449&gt;3.0.CO;2-N</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Jan R. Magnus</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>jan@janmagnus.nl</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Department of Econometrics &amp; OR, Tilburg University, Netherlands (emeritus; also VU Amsterdam)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Co-organizer of the coordinated 'experiment': multiple teams estimated the same model on shared data. J Applied Econometrics 12(5):459-465 (intro to special section). Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Magnus &amp; Morgan (1997) - The Experiment in Applied Econometrics (Tilburg Experiment: food demand / income elasticity)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/(SICI)1099-1255(199709/10)12:5&lt;459::AID-JAE449&gt;3.0.CO;2-N</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mary S. Morgan</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>m.morgan@lse.ac.uk</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Department of Economic History, London School of Economics, UK</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Co-organizer. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Ortloff et al. (2023) - Different Researchers, Different Results? Influence of Researcher Experience and Data Type During Qualitative Analysis (Security Advice)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3544548.3580766</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Anna-Marie Ortloff</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ortloff@cs.uni-bonn.de</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>University of Bonn, Germany (Behavioural Security Research Group)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Lead organizer. CHI 2023. Many independent coders/analysts qualitatively analyze the same security-advice interview/survey data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ortloff et al. (2023) - Different Researchers, Different Results? Influence of Researcher Experience and Data Type During Qualitative Analysis (Security Advice)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3544548.3580766</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Matthew Smith</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>University of Bonn &amp; Fraunhofer FKIE, Germany</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Senior PI. Email per uni-bonn pattern; verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Huber et al. (2023) - Competition and Moral Behavior: A Meta-analysis of Forty-Five Crowd-Sourced Experimental Designs</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2215572120</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Christoph Huber</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>christoph.huber@wu.ac.at</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Institute for Finance, Banking and Insurance, WU Vienna University of Economics and Business, Austria</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Lead organizer. PNAS 120(23):e2215572120. 45 research teams independently DESIGNED experiments for the same question (design many-analyst). Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Huber et al. (2023) - Competition and Moral Behavior: A Meta-analysis of Forty-Five Crowd-Sourced Experimental Designs</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2215572120</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Anna Dreber</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>anna.dreber@hhs.se</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Stockholm School of Economics, Sweden</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Huber et al. (2023) - Competition and Moral Behavior: A Meta-analysis of Forty-Five Crowd-Sourced Experimental Designs</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2215572120</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Juergen Huber</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>juergen.huber@uibk.ac.at</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>University of Innsbruck, Austria</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Huber et al. (2023) - Competition and Moral Behavior: A Meta-analysis of Forty-Five Crowd-Sourced Experimental Designs</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2215572120</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Magnus Johannesson</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>magnus.johannesson@hhs.se</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Stockholm School of Economics, Sweden</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Huber et al. (2023) - Competition and Moral Behavior: A Meta-analysis of Forty-Five Crowd-Sourced Experimental Designs</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.2215572120</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Michael Kirchler</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>michael.kirchler@uibk.ac.at</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>University of Innsbruck, Austria</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Coordinator.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete expansion passes: 24 many-analyst studies, 58 organizer rows
Adds EEGManyPipelines, Coretta (phonetics), Kowall (epidemiology), Salganik
(Fragile Families), van Dongen, and Starns; files Fillard, AI-analyst, Delios,
Rohrer, Aczel, and Kummerfeld as inappropriate. Recovers organizer emails
(down to 3 missing co-organizers). Finalizes PROGRESS log; queue empty.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,17 +742,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>E.M.Rinke@leeds.ac.uk</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>University of Leeds, UK (School of Politics and International Studies)</t>
+          <t>School of Politics and International Studies, University of Leeds, UK</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Co-organizer. Email to be confirmed.</t>
+          <t>Co-organizer (CRI).</t>
         </is>
       </c>
     </row>
@@ -774,17 +774,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>A.Wuttke@lmu.de</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>LMU Munich, Germany (Political Science)</t>
+          <t>Geschwister Scholl Institute of Political Science, LMU Munich, Germany</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Co-organizer. Email to be confirmed.</t>
+          <t>Co-organizer (CRI).</t>
         </is>
       </c>
     </row>
@@ -806,12 +806,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>jlandy@nova.edu</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Nova Southeastern University, FL, USA (Dept. of Psychology)</t>
+          <t>Department of Psychology and Neuroscience, Nova Southeastern University, FL, USA</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -870,17 +870,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>rotemb9@gmail.com</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Sagol School of Neuroscience, Tel Aviv University (at time of study); later Dartmouth College / Technion</t>
+          <t>Sagol School of Neuroscience, Tel Aviv University (study); later Dartmouth College; now Hebrew University of Jerusalem</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lead organizer of NARPS. Nature 582:84-88. 70 teams analyzed fMRI mixed-gamble data, 9 hypotheses. Email to verify.</t>
+          <t>Lead organizer of NARPS. Nature 582:84-88. 70 teams, fMRI mixed-gamble, 9 hypotheses.</t>
         </is>
       </c>
     </row>
@@ -1318,17 +1318,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>elliot.gould@unimelb.edu.au</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>School of BioSciences, University of Melbourne, Australia</t>
+          <t>School of Agriculture, Food and Ecosystem Sciences, University of Melbourne, Australia</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Co-lead author/organizer (they/them). BMC Biology 23:35. 174 analysts/teams, 2 datasets. Email: unimelb.edu.au domain, exact unconfirmed.</t>
+          <t>Co-lead organizer (they/them). BMC Biology 23:35.</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>hannahsfraser@gmail.com</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Co-lead author/organizer. Email unconfirmed (hannahsfraser@gmail.com likely).</t>
+          <t>Co-lead organizer (repliCATS / IMeRG).</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>ao2671@cumc.columbia.edu</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Department of Biomedical Informatics, Columbia University Irving Medical Center, NY, USA (now Johnson &amp; Johnson)</t>
+          <t>Department of Biomedical Informatics, Columbia University, NY, USA (now Johnson &amp; Johnson)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Lead organizer (OHDSI). JAMIA 30(5):859-868. 9 teams reproduce same observational study. Email to verify.</t>
+          <t>Lead organizer (OHDSI). Email per Columbia CUMC pattern; VERIFY prefix (ao2671).</t>
         </is>
       </c>
     </row>
@@ -1542,17 +1542,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>gilles.dutilh@usb.ch</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Department of Psychology, University of Basel, Switzerland (now University Hospital Basel)</t>
+          <t>Department of Clinical Research, University Hospital Basel, Switzerland</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Lead organizer. Psychonomic Bulletin &amp; Review 26(4):1051-1069. 17 teams analyzed same 14 RT datasets, blinded. Email to verify (unibas.ch/usb.ch).</t>
+          <t>Lead organizer. Psychon Bull Rev 26(4):1051-1069. 17 teams analyzed same 14 RT datasets, blinded.</t>
         </is>
       </c>
     </row>
@@ -1574,17 +1574,17 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
+          <t>Udo.Boehm@cwi.nl</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Department of Psychology, University of Amsterdam / University of Groningen, Netherlands</t>
+          <t>University of Amsterdam / CWI, Netherlands</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Lead organizer. J Mathematical Psychology 87:46-75. Multiple expert DDM teams each fit the same standardized data. Email to verify.</t>
+          <t>Lead organizer. J Math Psych 87:46-75. Multiple expert DDM teams fit the same standardized data.</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1766,18 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FAILED TO FIND</t>
-        </is>
-      </c>
+          <t>smith@cs.uni-bonn.de</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>University of Bonn &amp; Fraunhofer FKIE, Germany</t>
+          <t>Institute of Computer Science, University of Bonn &amp; Fraunhofer FKIE, Germany</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Senior PI. Email per uni-bonn pattern; verify.</t>
+          <t>Senior PI (Usable Security). Verify email.</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1930,6 @@
           <t>michael.kirchler@uibk.ac.at</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>University of Innsbruck, Austria</t>
@@ -1938,6 +1938,390 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>Coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Trubutschek et al. (2024) - EEGManyPipelines: A Large-scale, Grassroots Multi-analyst Study of EEG Analysis Practices in the Wild</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1162/jocn_a_02087</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Darinka Trubutschek</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>darinka.trubutschek@ae.mpg.de</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Max Planck Institute for Empirical Aesthetics, Frankfurt am Main, Germany</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Lead/corresponding organizer (steering committee, flat hierarchy). J Cog Neuro 36(2):217-240. 168 teams / 396 researchers analyzed same EEG dataset. Project email eegmanypipelines@gmail.com. Verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Trubutschek et al. (2024) - EEGManyPipelines: A Large-scale, Grassroots Multi-analyst Study of EEG Analysis Practices in the Wild</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1162/jocn_a_02087</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Niko A. Busch</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>niko.busch@uni-muenster.de</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Institute of Psychology, University of Munster, Germany</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Senior steering-committee organizer. Verify email pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Trubutschek et al. (2024) - EEGManyPipelines: A Large-scale, Grassroots Multi-analyst Study of EEG Analysis Practices in the Wild</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1162/jocn_a_02087</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Gustav Nilsonne</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>gustav.nilsonne@ki.se</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Department of Clinical Neuroscience, Karolinska Institutet, Stockholm, Sweden</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Senior steering-committee organizer. Verify email pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Coretta et al. (2023) - Multidimensional Signals and Analytic Flexibility: Estimating Degrees of Freedom in Human-Speech Analyses</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/25152459231162567</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Stefano Coretta</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>stefano.coretta@ed.ac.uk</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Linguistics and English Language, University of Edinburgh, UK</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Lead organizer. AMPPS (many-analyst phonetics; ~80 analysts/teams, same speech data). Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Kowall et al. (2025) - A Multi-Analyst Study on Marital Status and Cardiovascular Disease (SHARE data)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12874-025-02546-w</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Bernd Kowall</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>bernd.kowall@uk-essen.de</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Institute for Medical Informatics, Biometry and Epidemiology, University Hospital Essen, Germany</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Lead organizer. Multi-analyst study in epidemiology (marital status &amp; CVD, SHARE). DOI/venue to confirm. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Salganik et al. (2020) - Measuring the Predictability of Life Outcomes with a Scientific Mass Collaboration (Fragile Families Challenge)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.1915006117</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Matthew J. Salganik</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>mjs3@princeton.edu</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Department of Sociology, Princeton University, NJ, USA</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Lead organizer, Fragile Families Challenge (common-task mass collaboration: 160 teams predict same 6 outcomes from same data). PNAS 117(15):8398-8403. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Salganik et al. (2020) - Measuring the Predictability of Life Outcomes with a Scientific Mass Collaboration (Fragile Families Challenge)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.1915006117</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Ian Lundberg</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Princeton University (now UCLA), USA</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Co-organizer. Verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Salganik et al. (2020) - Measuring the Predictability of Life Outcomes with a Scientific Mass Collaboration (Fragile Families Challenge)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1073/pnas.1915006117</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sara McLanahan</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Princeton University, NJ, USA</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Co-organizer (Fragile Families PI). Verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>van Dongen et al. (2019) - Multiple Perspectives on Inference for Two Simple Statistical Scenarios</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/00031305.2019.1565553</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Noah N. N. van Dongen</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>n.n.n.vandongen@uva.nl</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Department of Psychology, University of Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Lead organizer. The American Statistician 73(S1):328-339. Multiple statistician teams analyze same two scenarios. Email per UvA pattern; verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>van Dongen et al. (2019) - Multiple Perspectives on Inference for Two Simple Statistical Scenarios</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/00031305.2019.1565553</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Eric-Jan Wagenmakers</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ej.wagenmakers@gmail.com</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Department of Psychological Methods, University of Amsterdam, Netherlands</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Senior co-organizer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Starns et al. (2019) - Assessing Theoretical Conclusions With Blinded Inference to Investigate a Potential Inference Crisis</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/2515245919869583</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Jeffrey J. Starns</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>jstarns@umass.edu</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Department of Psychological and Brain Sciences, University of Massachusetts Amherst, USA</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Lead/corresponding organizer. AMPPS 2(4):335-349. Many analyst teams use blinded inference on the same recognition-memory data. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Starns et al. (2019) - Assessing Theoretical Conclusions With Blinded Inference to Investigate a Potential Inference Crisis</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/2515245919869583</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Caren M. Rotello</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>rotello@umass.edu</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Department of Psychological and Brain Sciences, University of Massachusetts Amherst, USA</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Senior co-organizer. Verify email.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Round 3: process user-provided many-analyst list (+6 studies, 30 total)
Adds Multi100 (Aczel & Szaszi, Nature 2025), Maier-Hein 2017, Veronese 2021,
FIAC 2006, Fillard 2011 (moved from inappropriate), and Riemann 2003. Files
MAPS, Many Speech Analyses, Norgaard 2019, and the doc's commentary/perspective
pieces as inappropriate. Neuroimaging grand challenges now treated as in-scope
per the user's list. Broader post-2022 Scholar sweep found nothing new.
Regenerates CSV mirror; queue empty.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1769,7 +1769,6 @@
           <t>smith@cs.uni-bonn.de</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>Institute of Computer Science, University of Bonn &amp; Fraunhofer FKIE, Germany</t>
@@ -2322,6 +2321,263 @@
       <c r="G59" t="inlineStr">
         <is>
           <t>Senior co-organizer. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Aczel, Szaszi et al. (2025) - Multi100: Investigating the Analytical Robustness of the Social and Behavioural Sciences</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-025-09844-9</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Barnabas Szaszi</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>szaszi.barnabas@gmail.com</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Institute of Psychology, ELTE Eotvos Lorand University, Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Co-lead organizer, Multi100. Nature 652:135-142. ~246 analysts independently re-analyze 100 published social-science claims. Alt: szaszi.barnabas@ppk.elte.hu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Aczel, Szaszi et al. (2025) - Multi100: Investigating the Analytical Robustness of the Social and Behavioural Sciences</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-025-09844-9</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Balazs Aczel</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>aczel.balazs@ppk.elte.hu</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Institute of Psychology, ELTE Eotvos Lorand University, Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Co-lead/senior organizer, Multi100. Alt: balazs.aczel@gmail.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Maier-Hein et al. (2017) - The Challenge of Mapping the Human Connectome Based on Diffusion Tractography</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41467-017-01285-x</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Klaus H. Maier-Hein</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>k.maier-hein@dkfz.de</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Division of Medical Image Computing, German Cancer Research Center (DKFZ), Heidelberg, Germany</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Corresponding/senior organizer. Nature Communications 8:1349. 20 teams / 96 tractography pipelines on same diffusion-MRI data (ISMRM 2015 Tractography Challenge).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Veronese et al. (2021) - Reproducibility of Findings in Modern PET Neuroimaging: NRM2018 Grand Challenge</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/0271678X211015101</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Mattia Veronese</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>mattia.veronese@kcl.ac.uk</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Centre for Neuroimaging Sciences, IoPPN, King's College London, UK (also University of Padua)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Lead/corresponding organizer. J Cereb Blood Flow Metab. 14 international teams analyze same PET dataset (NRM2018 grand challenge).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>FIAC (2006) - Functional Imaging Analysis Contest: Reproducibility of fMRI Results Across Expert Analyses</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/hbm.20268</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Jean-Baptiste Poline</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>jean-baptiste.poline@mcgill.ca</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Montreal Neurological Institute, McGill University, Canada (formerly CEA/NeuroSpin, France)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Lead organizer. Human Brain Mapping 27(5) special issue. Multiple expert teams analyzed the same fMRI language dataset. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FIAC (2006) - Functional Imaging Analysis Contest: Reproducibility of fMRI Results Across Expert Analyses</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/hbm.20268</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Stephen C. Strother</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>sstrother@research.baycrest.org</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Rotman Research Institute, Baycrest &amp; University of Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Co-organizer. Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Fillard et al. (2011) - Quantitative Evaluation of 10 Tractography Algorithms on a Realistic Diffusion MR Phantom (Fiber Cup)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.neuroimage.2011.01.032</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Pierre Fillard</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>FAILED TO FIND</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Parietal Team, INRIA Saclay, France (later Therapixel)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Lead organizer (Fiber Cup challenge). NeuroImage 56(1):220-234. Multiple teams' tractography algorithms on same phantom data. Included per user's many-analyst list (was previously filed inappropriate). Verify email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Riemann (2003) - A Joint Project Against the Backdrop of a Research Tradition: Doing Biographical Research</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.17169/fqs-4.3.666</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Gerhard Riemann</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>gerhard.riemann@th-nuernberg.de</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Faculty of Social Sciences, Technische Hochschule Nurnberg (Georg-Simon-Ohm), Germany (Professor Emeritus)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Lead/organizer. FQS 4(3). Qualitative crowdsourcing: multiple researchers work the same biographical interview material (per user's many-analyst list). Emeritus; verify email.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Abstract and ManyAnalystStyle columns to Contact Info (all 30 studies)
Each study now carries a faithful abstract summary and a ManyAnalystStyle
write-up (scale, coordination/peer-review/blinding/platform features, the
point, and an interview-value flag for assessing the organizers). Adds
scripts/annotate.py helper; regenerates CSV mirror; updates PROGRESS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RCUvDYUjJHhdoT1mhhXgXA
</commit_message>
<xml_diff>
--- a/Contact Info.xlsx
+++ b/Contact Info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ManyAnalystStyle</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -489,6 +499,16 @@
           <t>Lead/corresponding author &amp; project organizer. Economic Inquiry 59(3):944-960. Seven replicators x two econ studies.</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Argues that the hundreds of unobserved data-preparation and analysis decisions researchers make ('researcher degrees of freedom') add uncertainty that standard errors do not capture. Using a many-analysts design, seven independent replicators each redid two published applied-microeconomics causal analyses, starting from raw public data. Replicators diverged widely in sample construction (no two had the same sample size) and in analysis; statistical significance varied and one effect even changed sign. The cross-replication standard deviation of estimates was 3-4x the mean reported standard error.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Small-but-deep design: 2 published econ studies x 7 independent replicators each (14 replications). Distinctive feature: replicators built the dataset from RAW data (most many-analyst studies hand out a pre-cleaned dataset), isolating data-cleaning as a variation source. Recruitment via U.S. department emails + Twitter; organizers coded each replicator's code line-by-line. Point: invisible data decisions, not just modeling, drive results. Interview value: HIGH - Huntington-Klein is a central repeat organizer (also led the 146-team Many-Economists project) with hands-on experience recruiting/coordinating economists and adjudicating their code.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +546,16 @@
           <t>Co-organizer (corresponding author). Forthcoming JEL. 146 research teams. Project: Many Economists Collaborative on Researcher Variation.</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Synthesizes the literature on 'researcher variation' and adds a large new many-analyst study in economics: 146 research teams estimated the same causal effect under progressively tighter constraints. Central estimates broadly agreed, but dispersion stayed substantial; imposing a shared research design actually reduced agreement (partly via adherence errors), while further constraining data cleaning improved it. Researcher variation is often as large as sampling uncertainty and is unevenly spread across research stages, implying conventional standard errors understate total uncertainty.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Large-scale: 146 teams, same causal question, with an experimental manipulation of how tightly the protocol constrained teams (free -&gt; shared design -&gt; shared data cleaning). Directly studies the EFFECT of organizer-imposed constraints on agreement - exactly the best-practices question. Preregistered; large collaborative roster ('Many-Economists Collaborative'). Interview value: VERY HIGH - Huntington-Klein &amp; Portner designed and ran one of the largest economics many-analyst projects and explicitly experimented with corralling tactics.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -558,6 +588,16 @@
           <t>Co-organizer. Also affiliated with Center for Studies in Demography and Ecology, Univ. of Washington. Personal site clausportner.com.</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Synthesizes the literature on 'researcher variation' and adds a large new many-analyst study in economics: 146 research teams estimated the same causal effect under progressively tighter constraints. Central estimates broadly agreed, but dispersion stayed substantial; imposing a shared research design actually reduced agreement (partly via adherence errors), while further constraining data cleaning improved it. Researcher variation is often as large as sampling uncertainty and is unevenly spread across research stages, implying conventional standard errors understate total uncertainty.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Large-scale: 146 teams, same causal question, with an experimental manipulation of how tightly the protocol constrained teams (free -&gt; shared design -&gt; shared data cleaning). Directly studies the EFFECT of organizer-imposed constraints on agreement - exactly the best-practices question. Preregistered; large collaborative roster ('Many-Economists Collaborative'). Interview value: VERY HIGH - Huntington-Klein &amp; Portner designed and ran one of the largest economics many-analyst projects and explicitly experimented with corralling tactics.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -590,6 +630,16 @@
           <t>Co-lead organizer. Adv Methods Practices Psych Sci 1(3):337-356. 29 teams analyzed soccer referee skin-tone/red-card data.</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>The original 'many analysts, one data set' study. 29 independent teams (61 analysts) used the same dataset to test whether soccer referees give more red cards to dark-skinned players. Analytic approaches and results varied widely - odds ratios from 0.89 to 2.93, with 20 teams finding a significant effect and 9 not - even after a peer-review stage among teams. Establishes that reasonable analytic choices materially affect conclusions.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>29 teams / 61 analysts, single shared dataset, one hypothesis. Foundational coordination template: teams first proposed analyses, then peer-reviewed each other's approaches and could revise; subjective beliefs were elicited. Organizers (Silberzahn, Uhlmann, Nosek) effectively created the field. Interview value: VERY HIGH - foundational organizers; Uhlmann has since run several crowdsourced projects (Schweinsberg, Landy).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -622,6 +672,16 @@
           <t>Co-lead/senior organizer.</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>The original 'many analysts, one data set' study. 29 independent teams (61 analysts) used the same dataset to test whether soccer referees give more red cards to dark-skinned players. Analytic approaches and results varied widely - odds ratios from 0.89 to 2.93, with 20 teams finding a significant effect and 9 not - even after a peer-review stage among teams. Establishes that reasonable analytic choices materially affect conclusions.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>29 teams / 61 analysts, single shared dataset, one hypothesis. Foundational coordination template: teams first proposed analyses, then peer-reviewed each other's approaches and could revise; subjective beliefs were elicited. Organizers (Silberzahn, Uhlmann, Nosek) effectively created the field. Interview value: VERY HIGH - foundational organizers; Uhlmann has since run several crowdsourced projects (Schweinsberg, Landy).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -654,6 +714,16 @@
           <t>Lead organizer. OBHDP 165:228-249. Crowdsourcing data analysis project (DataExplained).</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Independent analysts tested the same two hypotheses (effects of scientists' gender and status on verbosity in group discussions) on the same dataset; 29 analyses remained after exclusions. Results dispersed radically - from sizeable positive to sizeable negative effects - even though analysts were experienced and could see each other's work, with much of the variation traced to how analysts operationalized the constructs.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Many independent analyst teams on one dataset/two hypotheses (29 in final sample). Distinctive logistics: ran on the bespoke 'DataExplained' platform that captured analysts' analytic PATHS in real time, plus structured feedback/discussion rounds. Strong on tooling/operational infrastructure for tracking analysts. Interview value: HIGH - Schweinsberg + Uhlmann built custom infrastructure and managed deliberation; good source on tooling and operationalization.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -686,6 +756,16 @@
           <t>Senior/co-organizer.</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Independent analysts tested the same two hypotheses (effects of scientists' gender and status on verbosity in group discussions) on the same dataset; 29 analyses remained after exclusions. Results dispersed radically - from sizeable positive to sizeable negative effects - even though analysts were experienced and could see each other's work, with much of the variation traced to how analysts operationalized the constructs.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Many independent analyst teams on one dataset/two hypotheses (29 in final sample). Distinctive logistics: ran on the bespoke 'DataExplained' platform that captured analysts' analytic PATHS in real time, plus structured feedback/discussion rounds. Strong on tooling/operational infrastructure for tracking analysts. Interview value: HIGH - Schweinsberg + Uhlmann built custom infrastructure and managed deliberation; good source on tooling and operationalization.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -723,6 +803,16 @@
           <t>Lead organizer (CRI / Crowdsourced Replication Initiative). PNAS 119(44). 73 teams, immigration &amp; social policy support.</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>73 teams (161 researchers) independently tested the same hypothesis - whether immigration reduces support for social policy - on the same cross-national data. Numerical results ranged from strong negative to strong positive, and most of the dispersion could NOT be explained by teams' expertise, prior beliefs, or methodological choices, pointing to a large 'hidden universe' of idiosyncratic analytic variability.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Large: 73 teams / 161 researchers (the Crowdsourced Replication Initiative, CRI), one hypothesis, shared survey data. Multiple structured stages plus deliberation, and a systematic test of whether researcher characteristics explain variance. Heavily documented process. Interview value: VERY HIGH - Breznau/Rinke/Wuttke ran a very large social-science crowdsourcing effort and have written reflectively about recruitment, attrition, and coordination.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -755,6 +845,16 @@
           <t>Co-organizer (CRI).</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>73 teams (161 researchers) independently tested the same hypothesis - whether immigration reduces support for social policy - on the same cross-national data. Numerical results ranged from strong negative to strong positive, and most of the dispersion could NOT be explained by teams' expertise, prior beliefs, or methodological choices, pointing to a large 'hidden universe' of idiosyncratic analytic variability.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Large: 73 teams / 161 researchers (the Crowdsourced Replication Initiative, CRI), one hypothesis, shared survey data. Multiple structured stages plus deliberation, and a systematic test of whether researcher characteristics explain variance. Heavily documented process. Interview value: VERY HIGH - Breznau/Rinke/Wuttke ran a very large social-science crowdsourcing effort and have written reflectively about recruitment, attrition, and coordination.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -787,6 +887,16 @@
           <t>Co-organizer (CRI).</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>73 teams (161 researchers) independently tested the same hypothesis - whether immigration reduces support for social policy - on the same cross-national data. Numerical results ranged from strong negative to strong positive, and most of the dispersion could NOT be explained by teams' expertise, prior beliefs, or methodological choices, pointing to a large 'hidden universe' of idiosyncratic analytic variability.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Large: 73 teams / 161 researchers (the Crowdsourced Replication Initiative, CRI), one hypothesis, shared survey data. Multiple structured stages plus deliberation, and a systematic test of whether researcher characteristics explain variance. Heavily documented process. Interview value: VERY HIGH - Breznau/Rinke/Wuttke ran a very large social-science crowdsourcing effort and have written reflectively about recruitment, attrition, and coordination.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -819,6 +929,16 @@
           <t>Lead author. Psychological Bulletin 146(5):451-479. 15 teams designed studies for 5 hypotheses.</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Extends the many-analyst idea upstream to study DESIGN: 15 independent teams each designed studies and materials to test the same five research questions (moral judgment, negotiation, implicit cognition), and a large shared sample then ran all designs. Effect sizes varied dramatically - often significant in opposite directions across teams - showing that design choices, not just analysis, shape results.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>15 teams, but the variation is in study DESIGN ('crowdsourcing hypothesis tests'), a different flavor. Coordinating many designers and then fielding all their studies on one common participant pool is a sizeable logistical operation. Senior organizer Uhlmann (recurring). Interview value: HIGH - covers the design-stage organizing problem, complementary to analysis-only projects.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -851,6 +971,16 @@
           <t>Senior organizer (corresponding).</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Extends the many-analyst idea upstream to study DESIGN: 15 independent teams each designed studies and materials to test the same five research questions (moral judgment, negotiation, implicit cognition), and a large shared sample then ran all designs. Effect sizes varied dramatically - often significant in opposite directions across teams - showing that design choices, not just analysis, shape results.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>15 teams, but the variation is in study DESIGN ('crowdsourcing hypothesis tests'), a different flavor. Coordinating many designers and then fielding all their studies on one common participant pool is a sizeable logistical operation. Senior organizer Uhlmann (recurring). Interview value: HIGH - covers the design-stage organizing problem, complementary to analysis-only projects.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -883,6 +1013,16 @@
           <t>Lead organizer of NARPS. Nature 582:84-88. 70 teams, fMRI mixed-gamble, 9 hypotheses.</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>70 independent teams analyzed the same fMRI dataset to evaluate nine pre-specified hypotheses about brain activity in a gambling task. Reported yes/no hypothesis decisions varied substantially across teams (driven by pipeline choices such as smoothing and thresholding), and an accompanying prediction market showed peers over-estimated how replicable the results would be. A landmark demonstration of analytic variability in neuroimaging.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>70 teams / ~180 analysts, shared fMRI data, 9 pre-registered hypotheses with structured binary outputs. Sophisticated operational design: standardized result reporting plus a PREDICTION MARKET on outcomes. Multi-site senior team (Botvinik-Nezer, Schonberg, Poldrack, Nichols). Interview value: VERY HIGH - among the most organizationally complex many-analyst projects; strong on standardized reporting and incentive mechanisms.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -915,6 +1055,16 @@
           <t>Corresponding author / senior organizer.</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>70 independent teams analyzed the same fMRI dataset to evaluate nine pre-specified hypotheses about brain activity in a gambling task. Reported yes/no hypothesis decisions varied substantially across teams (driven by pipeline choices such as smoothing and thresholding), and an accompanying prediction market showed peers over-estimated how replicable the results would be. A landmark demonstration of analytic variability in neuroimaging.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>70 teams / ~180 analysts, shared fMRI data, 9 pre-registered hypotheses with structured binary outputs. Sophisticated operational design: standardized result reporting plus a PREDICTION MARKET on outcomes. Multi-site senior team (Botvinik-Nezer, Schonberg, Poldrack, Nichols). Interview value: VERY HIGH - among the most organizationally complex many-analyst projects; strong on standardized reporting and incentive mechanisms.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -947,6 +1097,16 @@
           <t>Corresponding author / senior organizer.</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>70 independent teams analyzed the same fMRI dataset to evaluate nine pre-specified hypotheses about brain activity in a gambling task. Reported yes/no hypothesis decisions varied substantially across teams (driven by pipeline choices such as smoothing and thresholding), and an accompanying prediction market showed peers over-estimated how replicable the results would be. A landmark demonstration of analytic variability in neuroimaging.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>70 teams / ~180 analysts, shared fMRI data, 9 pre-registered hypotheses with structured binary outputs. Sophisticated operational design: standardized result reporting plus a PREDICTION MARKET on outcomes. Multi-site senior team (Botvinik-Nezer, Schonberg, Poldrack, Nichols). Interview value: VERY HIGH - among the most organizationally complex many-analyst projects; strong on standardized reporting and incentive mechanisms.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -979,6 +1139,16 @@
           <t>Lead organizer. Journal of Finance 79(3):2339-2390. 164 teams test 6 finance hypotheses on same data. Organizing committee = first 8 authors (Menkveld, Dreber, Holzmeister, Huber, Johannesson, Kirchler, Razen, Weitzel).</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1011,6 +1181,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1043,6 +1223,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1075,6 +1265,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1107,6 +1307,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1139,6 +1349,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1171,6 +1391,16 @@
           <t>Organizing committee / research coordinator. Email to verify.</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1203,6 +1433,16 @@
           <t>Organizing committee / research coordinator.</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>164 research teams tested the same six hypotheses on the same financial-markets dataset. Dispersion across teams ('nonstandard errors') was sizeable - comparable to or exceeding standard errors. Crucially, a peer-review stage (teams' analyses were evaluated and could be revised) reduced dispersion, and the paper quantifies how much peer feedback tightens results.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Very large: 164 teams, 6 hypotheses, one dataset, run by an 8-person coordinating committee plus hundreds of analysts. Explicitly built in a PEER-REVIEW treatment and measured its effect on dispersion - directly an organizing 'best practice.' Massive coordination in finance. Interview value: VERY HIGH - Menkveld + the Innsbruck/SSE committee (Dreber, Holzmeister, Huber, Johannesson, Kirchler) are serial organizers of huge crowd studies with deep logistics expertise.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1235,6 +1475,16 @@
           <t>Lead organizer, Many-Analysts Religion Project (MARP). Religion Brain &amp; Behavior 13(3):237-283. 120+ analyst teams.</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>120 analysis teams used the same cross-national dataset (10,535 people, 24 countries) to answer two preregistered questions about the religiosity-well-being link. Effect sizes and conclusions varied, though most teams found a positive association; a companion strand compared analytic blinding versus preregistration as bias controls.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120 teams, shared multinational survey data, 2 questions. Methodologically rich operations: tested analysis-BLINDING vs preregistration, and elicited subjective evidence assessments. Run by the Amsterdam/ELTE metascience group (Hoogeveen, Sarafoglou, Aczel). Interview value: VERY HIGH - these organizers also wrote the field's consensus guidance for multi-analyst studies and built the SEES instrument; among the best positioned to speak to best practices.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1267,6 +1517,16 @@
           <t>Co-organizer, MARP.</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>120 analysis teams used the same cross-national dataset (10,535 people, 24 countries) to answer two preregistered questions about the religiosity-well-being link. Effect sizes and conclusions varied, though most teams found a positive association; a companion strand compared analytic blinding versus preregistration as bias controls.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120 teams, shared multinational survey data, 2 questions. Methodologically rich operations: tested analysis-BLINDING vs preregistration, and elicited subjective evidence assessments. Run by the Amsterdam/ELTE metascience group (Hoogeveen, Sarafoglou, Aczel). Interview value: VERY HIGH - these organizers also wrote the field's consensus guidance for multi-analyst studies and built the SEES instrument; among the best positioned to speak to best practices.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1299,6 +1559,16 @@
           <t>Co-organizer / senior, MARP. Alt: balazs.aczel@gmail.com.</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>120 analysis teams used the same cross-national dataset (10,535 people, 24 countries) to answer two preregistered questions about the religiosity-well-being link. Effect sizes and conclusions varied, though most teams found a positive association; a companion strand compared analytic blinding versus preregistration as bias controls.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120 teams, shared multinational survey data, 2 questions. Methodologically rich operations: tested analysis-BLINDING vs preregistration, and elicited subjective evidence assessments. Run by the Amsterdam/ELTE metascience group (Hoogeveen, Sarafoglou, Aczel). Interview value: VERY HIGH - these organizers also wrote the field's consensus guidance for multi-analyst studies and built the SEES instrument; among the best positioned to speak to best practices.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1331,6 +1601,16 @@
           <t>Co-lead organizer (they/them). BMC Biology 23:35.</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Two parallel many-analyst studies in ecology and evolutionary biology: independent analysts (174 in total across the two datasets) answered the same questions - on blue-tit nestling growth and on Eucalyptus seedling/grass cover - using the same data. Effect sizes and even directions varied widely, and analytic choices plus a peer-rating stage explained little of the deviation.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Two shared datasets, ~174 analysts/teams, with a structured peer-review rating of each analysis. Cross-disciplinary (SORTEE community) and heavily documented. Interview value: HIGH - Parker/Fraser/Gould ran a careful, well-documented ecology crowd study and are organized around reproducibility methods.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1363,6 +1643,16 @@
           <t>Co-lead organizer (repliCATS / IMeRG).</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Two parallel many-analyst studies in ecology and evolutionary biology: independent analysts (174 in total across the two datasets) answered the same questions - on blue-tit nestling growth and on Eucalyptus seedling/grass cover - using the same data. Effect sizes and even directions varied widely, and analytic choices plus a peer-rating stage explained little of the deviation.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Two shared datasets, ~174 analysts/teams, with a structured peer-review rating of each analysis. Cross-disciplinary (SORTEE community) and heavily documented. Interview value: HIGH - Parker/Fraser/Gould ran a careful, well-documented ecology crowd study and are organized around reproducibility methods.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1395,6 +1685,16 @@
           <t>Corresponding/senior organizer (SORTEE).</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Two parallel many-analyst studies in ecology and evolutionary biology: independent analysts (174 in total across the two datasets) answered the same questions - on blue-tit nestling growth and on Eucalyptus seedling/grass cover - using the same data. Effect sizes and even directions varied widely, and analytic choices plus a peer-rating stage explained little of the deviation.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Two shared datasets, ~174 analysts/teams, with a structured peer-review rating of each analysis. Cross-disciplinary (SORTEE community) and heavily documented. Interview value: HIGH - Parker/Fraser/Gould ran a careful, well-documented ecology crowd study and are organized around reproducibility methods.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1427,6 +1727,16 @@
           <t>Lead organizer (OHDSI). Email per Columbia CUMC pattern; VERIFY prefix (ao2671).</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Nine independent teams attempted to reproduce the SAME observational pharmaco-epidemiology study using a shared protocol and a common data model (OHDSI). Despite the shared task, teams made discordant design and implementation choices that produced different estimates, showing that even 'reproduction' of one study leaves substantial investigator discretion.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Smaller (9 teams) but distinctive: a shared, highly STRUCTURED protocol and common data model, so it studies discretion under heavy standardization. Run within the OHDSI network (Ostropolets, Hripcsak). Interview value: MEDIUM-HIGH - useful perspective on coordinating teams via rigorous shared protocols/infrastructure in medicine.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1459,6 +1769,16 @@
           <t>Senior/corresponding organizer (OHDSI).</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Nine independent teams attempted to reproduce the SAME observational pharmaco-epidemiology study using a shared protocol and a common data model (OHDSI). Despite the shared task, teams made discordant design and implementation choices that produced different estimates, showing that even 'reproduction' of one study leaves substantial investigator discretion.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Smaller (9 teams) but distinctive: a shared, highly STRUCTURED protocol and common data model, so it studies discretion under heavy standardization. Run within the OHDSI network (Ostropolets, Hripcsak). Interview value: MEDIUM-HIGH - useful perspective on coordinating teams via rigorous shared protocols/infrastructure in medicine.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1491,6 +1811,16 @@
           <t>Lead organizer. J Psychosomatic Research 137:110211. 12 research labs analyzed one patient's ESM time-series. Email per UMCG pattern; verify.</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>12 research teams analyzed the SAME single patient's experience-sampling (ESM) time-series to recommend clinical treatment targets. Teams selected widely different targets and offered different rationales, demonstrating that person-specific clinical inferences depend heavily on the analyst.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>12 teams, one shared single-subject clinical dataset, applied question (treatment targets). Clinically framed; modest scale but a clean design. Organizers Bastiaansen &amp; Bringmann (Groningen). Interview value: MEDIUM - solid organizer experience at small scale; strongest if clinical/idiographic applications are of interest.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1523,6 +1853,16 @@
           <t>Senior/corresponding organizer.</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>12 research teams analyzed the SAME single patient's experience-sampling (ESM) time-series to recommend clinical treatment targets. Teams selected widely different targets and offered different rationales, demonstrating that person-specific clinical inferences depend heavily on the analyst.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>12 teams, one shared single-subject clinical dataset, applied question (treatment targets). Clinically framed; modest scale but a clean design. Organizers Bastiaansen &amp; Bringmann (Groningen). Interview value: MEDIUM - solid organizer experience at small scale; strongest if clinical/idiographic applications are of interest.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1555,6 +1895,16 @@
           <t>Lead organizer. Psychon Bull Rev 26(4):1051-1069. 17 teams analyzed same 14 RT datasets, blinded.</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>17 teams each analyzed the same 14 two-condition response-time datasets while BLINDED to what had been manipulated, then inferred the underlying change using cognitive models of their choice. Conclusions were fairly consistent across teams, but 'modeler's degrees of freedom' affected inferences, and simpler methods often performed as well as complex ones.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>17 teams, 14 shared RT datasets, with a distinctive BLINDING design (teams did not know the ground-truth manipulation). Strong on blinded-analysis methodology. Organizer Dutilh. Interview value: MEDIUM - good on blinded-inference logistics within a specialist community.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1587,6 +1937,16 @@
           <t>Lead organizer. J Math Psych 87:46-75. Multiple expert DDM teams fit the same standardized data.</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>An expert-elicitation form of many-analyst work: multiple groups from the diffusion-decision-model community each applied their own fitting methods to the same standardized data to estimate notoriously hard 'across-trial variability' parameters, then distilled collective advice. Estimates were highly uncertain across experts, and the paper issues consensus recommendations.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Expert-elicitation flavor: a set of DDM modeling labs each fit shared data, organized into collective recommendations. Smaller, specialist community; senior organizers Boehm &amp; Wagenmakers (Amsterdam). Interview value: MEDIUM - niche but a clean example of corralling method experts toward consensus.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1619,6 +1979,16 @@
           <t>Senior organizer.</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>An expert-elicitation form of many-analyst work: multiple groups from the diffusion-decision-model community each applied their own fitting methods to the same standardized data to estimate notoriously hard 'across-trial variability' parameters, then distilled collective advice. Estimates were highly uncertain across experts, and the paper issues consensus recommendations.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Expert-elicitation flavor: a set of DDM modeling labs each fit shared data, organized into collective recommendations. Smaller, specialist community; senior organizers Boehm &amp; Wagenmakers (Amsterdam). Interview value: MEDIUM - niche but a clean example of corralling method experts toward consensus.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1651,6 +2021,16 @@
           <t>Journalistic many-analyst: 4 pollster teams analyzed the same 2016 Florida poll raw data. Organizer/author Nate Cohn. Email per NYT firstname.lastname@nytimes.com pattern; verify.</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>A journalistic many-analyst demonstration: the New York Times Upshot gave the same raw 2016 Florida presidential poll to four respected pollsters, who produced four different topline results (about a 4-point spread) because of differing weighting and likely-voter choices. Illustrates analyst discretion in a real polling context.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Only 4 analysts/teams, one shared raw dataset, non-academic. A vivid, public-facing illustration but a light-touch organizing effort (a journalist commissioning four pollsters). Contact is a journalist, not a researcher. Interview value: LOWER for best-practices logistics, though useful for the communication/illustration angle.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1683,6 +2063,16 @@
           <t>Co-organizer of the coordinated 'experiment': multiple teams estimated the same model on shared data. J Applied Econometrics 12(5):459-465 (intro to special section). Verify email.</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>An early coordinated 'experiment in applied econometrics': several invited teams of econometricians independently analyzed the same data following a shared brief, to expose how method choices drive empirical conclusions. A 1990s precursor to modern many-analyst studies, organized as a deliberate special-issue experiment.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Historic precursor (1990s): multiple invited expert teams, shared data and task, coordinated by Magnus &amp; Morgan as a deliberate 'experiment.' Small by modern standards and dated, but the organizers pioneered the format. Interview value: MEDIUM-LOWER - historically insightful but old; organizers senior/emeritus.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1715,6 +2105,16 @@
           <t>Co-organizer. Verify email.</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>An early coordinated 'experiment in applied econometrics': several invited teams of econometricians independently analyzed the same data following a shared brief, to expose how method choices drive empirical conclusions. A 1990s precursor to modern many-analyst studies, organized as a deliberate special-issue experiment.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Historic precursor (1990s): multiple invited expert teams, shared data and task, coordinated by Magnus &amp; Morgan as a deliberate 'experiment.' Small by modern standards and dated, but the organizers pioneered the format. Interview value: MEDIUM-LOWER - historically insightful but old; organizers senior/emeritus.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1747,6 +2147,16 @@
           <t>Lead organizer. CHI 2023. Many independent coders/analysts qualitatively analyze the same security-advice interview/survey data.</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>A many-analyst study of QUALITATIVE research: multiple coders/analysts who varied in experience independently analyzed the same interview and survey data on security advice, showing that qualitative coding outcomes depend on researcher experience and on data type. Extends analytic-variability concerns to qualitative methods.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Qualitative many-analyst (independent coding of the same data), with a designed comparison across researcher experience levels. Distinct domain (HCI/usable security). Organizers Ortloff &amp; Smith (Bonn). Interview value: MEDIUM - valuable if best-practices scope includes qualitative coding; otherwise niche.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1779,6 +2189,16 @@
           <t>Senior PI (Usable Security). Verify email.</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>A many-analyst study of QUALITATIVE research: multiple coders/analysts who varied in experience independently analyzed the same interview and survey data on security advice, showing that qualitative coding outcomes depend on researcher experience and on data type. Extends analytic-variability concerns to qualitative methods.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Qualitative many-analyst (independent coding of the same data), with a designed comparison across researcher experience levels. Distinct domain (HCI/usable security). Organizers Ortloff &amp; Smith (Bonn). Interview value: MEDIUM - valuable if best-practices scope includes qualitative coding; otherwise niche.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1811,6 +2231,16 @@
           <t>Lead organizer. PNAS 120(23):e2215572120. 45 research teams independently DESIGNED experiments for the same question (design many-analyst). Verify email.</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>A design-stage crowd study: 45 independent research teams each designed an experiment to test the same question - does competition erode moral behavior? - and all designs were fielded on a large shared participant pool (&gt;18,000). Effect sizes varied with design choices, and the pooled evidence showed a small negative effect of competition on morality.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>45 teams, varying experimental DESIGN (design heterogeneity) rather than analysis; &gt;18k participants fielded across designs is substantial logistics. Run by the Innsbruck/SSE crowd-science group (Christoph Huber, Dreber, Johannesson, Kirchler). Interview value: HIGH - serial crowd-study organizers; complements analysis-only projects with design-stage organizing.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1843,6 +2273,16 @@
           <t>Coordinator.</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>A design-stage crowd study: 45 independent research teams each designed an experiment to test the same question - does competition erode moral behavior? - and all designs were fielded on a large shared participant pool (&gt;18,000). Effect sizes varied with design choices, and the pooled evidence showed a small negative effect of competition on morality.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>45 teams, varying experimental DESIGN (design heterogeneity) rather than analysis; &gt;18k participants fielded across designs is substantial logistics. Run by the Innsbruck/SSE crowd-science group (Christoph Huber, Dreber, Johannesson, Kirchler). Interview value: HIGH - serial crowd-study organizers; complements analysis-only projects with design-stage organizing.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1875,6 +2315,16 @@
           <t>Coordinator.</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>A design-stage crowd study: 45 independent research teams each designed an experiment to test the same question - does competition erode moral behavior? - and all designs were fielded on a large shared participant pool (&gt;18,000). Effect sizes varied with design choices, and the pooled evidence showed a small negative effect of competition on morality.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>45 teams, varying experimental DESIGN (design heterogeneity) rather than analysis; &gt;18k participants fielded across designs is substantial logistics. Run by the Innsbruck/SSE crowd-science group (Christoph Huber, Dreber, Johannesson, Kirchler). Interview value: HIGH - serial crowd-study organizers; complements analysis-only projects with design-stage organizing.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1907,6 +2357,16 @@
           <t>Coordinator.</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>A design-stage crowd study: 45 independent research teams each designed an experiment to test the same question - does competition erode moral behavior? - and all designs were fielded on a large shared participant pool (&gt;18,000). Effect sizes varied with design choices, and the pooled evidence showed a small negative effect of competition on morality.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>45 teams, varying experimental DESIGN (design heterogeneity) rather than analysis; &gt;18k participants fielded across designs is substantial logistics. Run by the Innsbruck/SSE crowd-science group (Christoph Huber, Dreber, Johannesson, Kirchler). Interview value: HIGH - serial crowd-study organizers; complements analysis-only projects with design-stage organizing.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1939,6 +2399,16 @@
           <t>Coordinator.</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>A design-stage crowd study: 45 independent research teams each designed an experiment to test the same question - does competition erode moral behavior? - and all designs were fielded on a large shared participant pool (&gt;18,000). Effect sizes varied with design choices, and the pooled evidence showed a small negative effect of competition on morality.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>45 teams, varying experimental DESIGN (design heterogeneity) rather than analysis; &gt;18k participants fielded across designs is substantial logistics. Run by the Innsbruck/SSE crowd-science group (Christoph Huber, Dreber, Johannesson, Kirchler). Interview value: HIGH - serial crowd-study organizers; complements analysis-only projects with design-stage organizing.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1971,6 +2441,16 @@
           <t>Lead/corresponding organizer (steering committee, flat hierarchy). J Cog Neuro 36(2):217-240. 168 teams / 396 researchers analyzed same EEG dataset. Project email eegmanypipelines@gmail.com. Verify.</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>168 analyst teams (396 researchers) independently analyzed the same EEG dataset to test the same predefined hypotheses, each with a pipeline they deemed appropriate. No two pipelines were identical and statistical conclusions varied substantially, quantifying analytic flexibility in EEG. A grassroots, community-run effort.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Very large (168 teams / 396 people), shared EEG data, predefined hypotheses. Notable governance: an explicitly FLAT steering committee, grassroots recruitment, and standardized result submission. A strong example of running a huge volunteer collaboration. Interview value: VERY HIGH - Trubutschek/Busch/Nilsonne coordinated a massive grassroots project and have described the organizational model in print.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2003,6 +2483,16 @@
           <t>Senior steering-committee organizer. Verify email pattern.</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>168 analyst teams (396 researchers) independently analyzed the same EEG dataset to test the same predefined hypotheses, each with a pipeline they deemed appropriate. No two pipelines were identical and statistical conclusions varied substantially, quantifying analytic flexibility in EEG. A grassroots, community-run effort.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Very large (168 teams / 396 people), shared EEG data, predefined hypotheses. Notable governance: an explicitly FLAT steering committee, grassroots recruitment, and standardized result submission. A strong example of running a huge volunteer collaboration. Interview value: VERY HIGH - Trubutschek/Busch/Nilsonne coordinated a massive grassroots project and have described the organizational model in print.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2035,6 +2525,16 @@
           <t>Senior steering-committee organizer. Verify email pattern.</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>168 analyst teams (396 researchers) independently analyzed the same EEG dataset to test the same predefined hypotheses, each with a pipeline they deemed appropriate. No two pipelines were identical and statistical conclusions varied substantially, quantifying analytic flexibility in EEG. A grassroots, community-run effort.</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Very large (168 teams / 396 people), shared EEG data, predefined hypotheses. Notable governance: an explicitly FLAT steering committee, grassroots recruitment, and standardized result submission. A strong example of running a huge volunteer collaboration. Interview value: VERY HIGH - Trubutschek/Busch/Nilsonne coordinated a massive grassroots project and have described the organizational model in print.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2067,6 +2567,16 @@
           <t>Lead organizer. AMPPS (many-analyst phonetics; ~80 analysts/teams, same speech data). Verify email.</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>The 'Many Speech Analyses' project: 46 analysts/teams independently analyzed the same speech-production dataset to answer the same phonetics question, with each team also peer-reviewing others. Reported effect sizes varied substantially, demonstrating analytic flexibility in both measurement and statistics in the speech sciences.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>46 teams, shared speech data, one question, with a built-in cross-team PEER-REVIEW stage; published as a Registered Report. Organizers Coretta/Casillas/Roettger also wrote a separate 'lessons learned in managing many-analyst projects' paper. Interview value: HIGH - organizers have explicitly reflected in print on research-management logistics.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2099,6 +2609,16 @@
           <t>Lead organizer. Multi-analyst study in epidemiology (marital status &amp; CVD, SHARE). DOI/venue to confirm. Verify email.</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Brings the multi-analyst approach to epidemiology: 16 analyst groups (24 researchers) independently analyzed the same SHARE cohort data to estimate the effect of marital status on cardiovascular disease. Estimates varied in size and sometimes direction, showing analytic variability in observational epidemiology.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>16 groups / 24 researchers, shared cohort data, one epidemiological question. Clean, recent, in a field new to many-analyst methods. Organizer Kowall (Essen). Interview value: MEDIUM-HIGH - a fresh organizer perspective bringing the method to epidemiology, at modest scale.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2131,6 +2651,16 @@
           <t>Lead organizer, Fragile Families Challenge (common-task mass collaboration: 160 teams predict same 6 outcomes from same data). PNAS 117(15):8398-8403. Verify email.</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>A 'common task' mass collaboration: 160 teams built predictive models for the same six life outcomes using the same rich longitudinal data (the Fragile Families study). Even the best models predicted poorly and barely beat a simple benchmark, and very different methods produced similarly limited accuracy - an unusually large, infrastructure-heavy collaboration.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Very large (160 teams), shared data, common PREDICTION task (not hypothesis testing). Ran like a structured data-science challenge with a submission platform, holdout scoring, and a coordinated special issue - serious operational machinery. Organizer Salganik (Princeton). Interview value: HIGH - distinctive expertise running large common-task challenges (platform, scoring, mass coordination).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2163,6 +2693,16 @@
           <t>Co-organizer. Verify.</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>A 'common task' mass collaboration: 160 teams built predictive models for the same six life outcomes using the same rich longitudinal data (the Fragile Families study). Even the best models predicted poorly and barely beat a simple benchmark, and very different methods produced similarly limited accuracy - an unusually large, infrastructure-heavy collaboration.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Very large (160 teams), shared data, common PREDICTION task (not hypothesis testing). Ran like a structured data-science challenge with a submission platform, holdout scoring, and a coordinated special issue - serious operational machinery. Organizer Salganik (Princeton). Interview value: HIGH - distinctive expertise running large common-task challenges (platform, scoring, mass coordination).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2195,6 +2735,16 @@
           <t>Co-organizer (Fragile Families PI). Verify.</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>A 'common task' mass collaboration: 160 teams built predictive models for the same six life outcomes using the same rich longitudinal data (the Fragile Families study). Even the best models predicted poorly and barely beat a simple benchmark, and very different methods produced similarly limited accuracy - an unusually large, infrastructure-heavy collaboration.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Very large (160 teams), shared data, common PREDICTION task (not hypothesis testing). Ran like a structured data-science challenge with a submission platform, holdout scoring, and a coordinated special issue - serious operational machinery. Organizer Salganik (Princeton). Interview value: HIGH - distinctive expertise running large common-task challenges (platform, scoring, mass coordination).</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2227,6 +2777,16 @@
           <t>Lead organizer. The American Statistician 73(S1):328-339. Multiple statistician teams analyze same two scenarios. Email per UvA pattern; verify.</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Four teams working in different statistical traditions (e.g., frequentist, Bayesian, likelihood) independently analyzed the same two simple datasets (a two-proportion comparison and a correlation). Numerical conclusions largely agreed, but interpretations and framework debates persisted - an illustration of analyst variability even on simple problems.</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Small (4 teams), shared simple data, focused on statistical-framework differences. Light logistical lift. Organizers van Dongen &amp; Wagenmakers (Amsterdam). Interview value: LOWER - small and pedagogical, though Wagenmakers is a recurring figure.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2259,6 +2819,16 @@
           <t>Senior co-organizer.</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Four teams working in different statistical traditions (e.g., frequentist, Bayesian, likelihood) independently analyzed the same two simple datasets (a two-proportion comparison and a correlation). Numerical conclusions largely agreed, but interpretations and framework debates persisted - an illustration of analyst variability even on simple problems.</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Small (4 teams), shared simple data, focused on statistical-framework differences. Light logistical lift. Organizers van Dongen &amp; Wagenmakers (Amsterdam). Interview value: LOWER - small and pedagogical, though Wagenmakers is a recurring figure.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2291,6 +2861,16 @@
           <t>Lead/corresponding organizer. AMPPS 2(4):335-349. Many analyst teams use blinded inference on the same recognition-memory data. Verify email.</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Multiple independent modeling teams analyzed the same recognition-memory data using their own cognitive models, with the data-generating conditions BLINDED, to test whether experts reach consistent theoretical conclusions. Modeling strategies varied greatly though conclusions were often similar, and reported quantities were highly variable, hinting at an 'inference crisis.'</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Many cognitive-modeling teams (a large author roster), shared data, with a blinded-inference design. Domain-specific (mathematical psychology). Organizers Starns &amp; Rotello (UMass). Interview value: MEDIUM - a good blinded-inference example within a specialist community.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2323,6 +2903,16 @@
           <t>Senior co-organizer. Verify email.</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Multiple independent modeling teams analyzed the same recognition-memory data using their own cognitive models, with the data-generating conditions BLINDED, to test whether experts reach consistent theoretical conclusions. Modeling strategies varied greatly though conclusions were often similar, and reported quantities were highly variable, hinting at an 'inference crisis.'</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Many cognitive-modeling teams (a large author roster), shared data, with a blinded-inference design. Domain-specific (mathematical psychology). Organizers Starns &amp; Rotello (UMass). Interview value: MEDIUM - a good blinded-inference example within a specialist community.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2355,6 +2945,16 @@
           <t>Co-lead organizer, Multi100. Nature 652:135-142. ~246 analysts independently re-analyze 100 published social-science claims. Alt: szaszi.barnabas@ppk.elte.hu.</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>The largest-scale analytic-robustness project to date: 246 analysts independently re-analyzed 100 already-published social-science claims (each claim re-analyzed by multiple analysts) to test whether independent experts reproduce the original conclusion and effect size. A substantial share of re-analyses diverged from the originals, quantifying analytic robustness across the social sciences.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Massive and structurally different: 100 papers x multiple independent analysts (246 total), coordinated centrally with strict workflows (matching analysts to papers, standardizing outputs across 100 claims). Organizers Aczel &amp; Szaszi (ELTE) are also authors of the field's consensus-guidance paper. Interview value: VERY HIGH - arguably the most ambitious coordination effort; organizers are methodology leaders for multi-analyst best practice.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2387,6 +2987,16 @@
           <t>Co-lead/senior organizer, Multi100. Alt: balazs.aczel@gmail.com.</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>The largest-scale analytic-robustness project to date: 246 analysts independently re-analyzed 100 already-published social-science claims (each claim re-analyzed by multiple analysts) to test whether independent experts reproduce the original conclusion and effect size. A substantial share of re-analyses diverged from the originals, quantifying analytic robustness across the social sciences.</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Massive and structurally different: 100 papers x multiple independent analysts (246 total), coordinated centrally with strict workflows (matching analysts to papers, standardizing outputs across 100 claims). Organizers Aczel &amp; Szaszi (ELTE) are also authors of the field's consensus-guidance paper. Interview value: VERY HIGH - arguably the most ambitious coordination effort; organizers are methodology leaders for multi-analyst best practice.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2419,6 +3029,16 @@
           <t>Corresponding/senior organizer. Nature Communications 8:1349. 20 teams / 96 tractography pipelines on same diffusion-MRI data (ISMRM 2015 Tractography Challenge).</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>A diffusion-MRI tractography 'challenge': 20 research groups submitted 96 different pipelines to reconstruct the same simulated brain white-matter connections from shared data with known ground truth. The reconstructions contained large proportions of invalid/false-positive bundles, revealing how strongly method choices affect connectome mapping.</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Challenge format: 20 groups / 96 submissions, shared data with ground truth, organized by Maier-Hein (DKFZ). Algorithm-comparison flavor (pipelines/methods rather than free analytic decisions). Interview value: MEDIUM - large and well-run, but a benchmark-challenge model; relevant if challenge-style organizing is of interest.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2451,6 +3071,16 @@
           <t>Lead/corresponding organizer. J Cereb Blood Flow Metab. 14 international teams analyze same PET dataset (NRM2018 grand challenge).</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>The NRM2018 PET 'grand challenge': 14 international teams analyzed the same PET neuroimaging dataset (with known ground truth) to quantify a tracer outcome, revealing variability in results across standard analysis pipelines and informing reproducibility in molecular imaging.</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>14 teams, shared PET data with known ground truth, challenge format at a conference. Organizer Veronese (KCL). Interview value: MEDIUM - a solid challenge-style example at moderate scale.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2483,6 +3113,16 @@
           <t>Lead organizer. Human Brain Mapping 27(5) special issue. Multiple expert teams analyzed the same fMRI language dataset. Verify email.</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>An early fMRI 'analysis contest': multiple expert teams independently analyzed the same functional-MRI language dataset with their own methods and software, and a synthesis paper compared the reproducibility of results across expert analyses. A pioneering 2005-06 precursor to NARPS.</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Historic precursor: several expert teams, shared fMRI data, organized as a contest with a synthesis paper (Poline, Strother et al.). Dated and modest scale. Interview value: MEDIUM-LOWER - pioneering but old; organizers (Poline, Strother) remain active in neuroimaging methods.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2515,6 +3155,16 @@
           <t>Co-organizer. Verify email.</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>An early fMRI 'analysis contest': multiple expert teams independently analyzed the same functional-MRI language dataset with their own methods and software, and a synthesis paper compared the reproducibility of results across expert analyses. A pioneering 2005-06 precursor to NARPS.</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Historic precursor: several expert teams, shared fMRI data, organized as a contest with a synthesis paper (Poline, Strother et al.). Dated and modest scale. Interview value: MEDIUM-LOWER - pioneering but old; organizers (Poline, Strother) remain active in neuroimaging methods.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2547,6 +3197,16 @@
           <t>Lead organizer (Fiber Cup challenge). NeuroImage 56(1):220-234. Multiple teams' tractography algorithms on same phantom data. Included per user's many-analyst list (was previously filed inappropriate). Verify email.</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>The 'Fiber Cup' tractography challenge: 10 tractography algorithms/teams were quantitatively evaluated on the same realistic diffusion-MRI phantom with known ground-truth fibers, comparing reconstruction accuracy across methods to benchmark the field.</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Challenge/benchmark format: ~10 algorithms/teams, shared phantom data with ground truth, organized by Fillard (INRIA). Method-comparison flavor. Interview value: MEDIUM-LOWER - benchmark-style; relevant only if challenge organizing is in scope.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2569,7 +3229,6 @@
           <t>gerhard.riemann@th-nuernberg.de</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>Faculty of Social Sciences, Technische Hochschule Nurnberg (Georg-Simon-Ohm), Germany (Professor Emeritus)</t>
@@ -2578,6 +3237,16 @@
       <c r="G67" t="inlineStr">
         <is>
           <t>Lead/organizer. FQS 4(3). Qualitative crowdsourcing: multiple researchers work the same biographical interview material (per user's many-analyst list). Emeritus; verify email.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Introduces a joint qualitative research project in which multiple researchers, within a shared biographical-research tradition, collectively worked the same biographical/interview materials - an early example of crowdsourced qualitative analysis and interpretive variability and consensus-building.</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Qualitative and collaborative (German biographical-research tradition); multiple researchers interpret shared material, more consensus-oriented than independent-team comparison. Small, old, qualitative. Organizer Riemann (emeritus). Interview value: LOWER - borderline fit; mainly of interest for the history of qualitative crowdsourcing.</t>
         </is>
       </c>
     </row>

</xml_diff>